<commit_message>
data: auto-fetch & update sentiment data up to 2026-08-24 (sentiment: 55.80)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -15269,6 +15269,9 @@
       <c r="D465">
         <v>45.13</v>
       </c>
+      <c r="E465">
+        <v>843.75</v>
+      </c>
       <c r="F465">
         <v>1.39</v>
       </c>
@@ -15278,8 +15281,11 @@
       <c r="H465">
         <v>49.21</v>
       </c>
+      <c r="I465">
+        <v>99.8</v>
+      </c>
       <c r="J465">
-        <v>41.14</v>
+        <v>55.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-08-24 (sentiment: 31.70)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -5746,10 +5746,10 @@
         <v>51.79</v>
       </c>
       <c r="I167">
-        <v>51.39</v>
+        <v>51.79</v>
       </c>
       <c r="J167">
-        <v>44.35</v>
+        <v>44.44</v>
       </c>
     </row>
     <row r="168" spans="1:10">
@@ -15270,7 +15270,7 @@
         <v>45.13</v>
       </c>
       <c r="E465">
-        <v>843.75</v>
+        <v>8.44</v>
       </c>
       <c r="F465">
         <v>1.39</v>
@@ -15282,10 +15282,10 @@
         <v>49.21</v>
       </c>
       <c r="I465">
-        <v>99.8</v>
+        <v>3.37</v>
       </c>
       <c r="J465">
-        <v>55.8</v>
+        <v>31.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-08-25 (sentiment: 29.96)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J465"/>
+  <dimension ref="A1:J466"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -15288,6 +15288,38 @@
         <v>31.7</v>
       </c>
     </row>
+    <row r="466" spans="1:10">
+      <c r="A466" s="2">
+        <v>46259.66666666666</v>
+      </c>
+      <c r="B466">
+        <v>1.4</v>
+      </c>
+      <c r="C466">
+        <v>42</v>
+      </c>
+      <c r="D466">
+        <v>46.5</v>
+      </c>
+      <c r="E466">
+        <v>6.95</v>
+      </c>
+      <c r="F466">
+        <v>0.6</v>
+      </c>
+      <c r="G466">
+        <v>67.66</v>
+      </c>
+      <c r="H466">
+        <v>51.39</v>
+      </c>
+      <c r="I466">
+        <v>0.2</v>
+      </c>
+      <c r="J466">
+        <v>29.96</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-08-28 (sentiment: 17.51)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J468"/>
+  <dimension ref="A1:J469"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15410,7 +15410,7 @@
         <v>58.5</v>
       </c>
       <c r="E468" t="n">
-        <v>5.89</v>
+        <v>7.57</v>
       </c>
       <c r="F468" t="n">
         <v>2.98</v>
@@ -15422,10 +15422,42 @@
         <v>65.48</v>
       </c>
       <c r="I468" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J468" t="n">
+        <v>17.41</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="2" t="n">
+        <v>46262.66666666666</v>
+      </c>
+      <c r="B469" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="C469" t="n">
+        <v>20.04</v>
+      </c>
+      <c r="D469" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="E469" t="n">
+        <v>7.63</v>
+      </c>
+      <c r="F469" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="G469" t="n">
         <v>0.2</v>
       </c>
-      <c r="J468" t="n">
-        <v>17.21</v>
+      <c r="H469" t="n">
+        <v>65.28</v>
+      </c>
+      <c r="I469" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="J469" t="n">
+        <v>17.51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-01 (sentiment: 33.58)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J470"/>
+  <dimension ref="A1:J471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15474,7 +15474,7 @@
         <v>58.5</v>
       </c>
       <c r="E470" t="n">
-        <v>7.12</v>
+        <v>7.16</v>
       </c>
       <c r="F470" t="n">
         <v>3.37</v>
@@ -15490,6 +15490,38 @@
       </c>
       <c r="J470" t="n">
         <v>34.47</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="2" t="n">
+        <v>46266.66666666666</v>
+      </c>
+      <c r="B471" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="C471" t="n">
+        <v>41.75</v>
+      </c>
+      <c r="D471" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="E471" t="n">
+        <v>7.48</v>
+      </c>
+      <c r="F471" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="G471" t="n">
+        <v>64.48</v>
+      </c>
+      <c r="H471" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="I471" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J471" t="n">
+        <v>33.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-02 (sentiment: 32.39)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J471"/>
+  <dimension ref="A1:J472"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15506,7 +15506,7 @@
         <v>58.5</v>
       </c>
       <c r="E471" t="n">
-        <v>7.48</v>
+        <v>6.86</v>
       </c>
       <c r="F471" t="n">
         <v>3.57</v>
@@ -15518,10 +15518,42 @@
         <v>65.67</v>
       </c>
       <c r="I471" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="J471" t="n">
-        <v>33.58</v>
+        <v>33.48</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="2" t="n">
+        <v>46267.66666666666</v>
+      </c>
+      <c r="B472" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="C472" t="n">
+        <v>40.51</v>
+      </c>
+      <c r="D472" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="E472" t="n">
+        <v>7.77</v>
+      </c>
+      <c r="F472" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="G472" t="n">
+        <v>58.93</v>
+      </c>
+      <c r="H472" t="n">
+        <v>65.48</v>
+      </c>
+      <c r="I472" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="J472" t="n">
+        <v>32.39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-03 (sentiment: 33.58)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J472"/>
+  <dimension ref="A1:J473"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15538,7 +15538,7 @@
         <v>58.5</v>
       </c>
       <c r="E472" t="n">
-        <v>7.77</v>
+        <v>6.64</v>
       </c>
       <c r="F472" t="n">
         <v>3.77</v>
@@ -15550,10 +15550,42 @@
         <v>65.48</v>
       </c>
       <c r="I472" t="n">
-        <v>1.39</v>
+        <v>0.2</v>
       </c>
       <c r="J472" t="n">
-        <v>32.39</v>
+        <v>32.09</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="2" t="n">
+        <v>46268.66666666666</v>
+      </c>
+      <c r="B473" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="C473" t="n">
+        <v>41.73</v>
+      </c>
+      <c r="D473" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="E473" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="F473" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="G473" t="n">
+        <v>64.09</v>
+      </c>
+      <c r="H473" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="I473" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J473" t="n">
+        <v>33.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-04 (sentiment: 33.28)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J473"/>
+  <dimension ref="A1:J474"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15570,7 +15570,7 @@
         <v>58.5</v>
       </c>
       <c r="E473" t="n">
-        <v>6.78</v>
+        <v>6.76</v>
       </c>
       <c r="F473" t="n">
         <v>3.97</v>
@@ -15586,6 +15586,38 @@
       </c>
       <c r="J473" t="n">
         <v>33.58</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="2" t="n">
+        <v>46269.66666666666</v>
+      </c>
+      <c r="B474" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="C474" t="n">
+        <v>41.57</v>
+      </c>
+      <c r="D474" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="E474" t="n">
+        <v>5.86</v>
+      </c>
+      <c r="F474" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="G474" t="n">
+        <v>63.29</v>
+      </c>
+      <c r="H474" t="n">
+        <v>65.48</v>
+      </c>
+      <c r="I474" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J474" t="n">
+        <v>33.28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-07 (sentiment: 34.77)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J474"/>
+  <dimension ref="A1:J475"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15602,7 +15602,7 @@
         <v>58.5</v>
       </c>
       <c r="E474" t="n">
-        <v>5.86</v>
+        <v>6.57</v>
       </c>
       <c r="F474" t="n">
         <v>4.17</v>
@@ -15618,6 +15618,38 @@
       </c>
       <c r="J474" t="n">
         <v>33.28</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="2" t="n">
+        <v>46272.66666666666</v>
+      </c>
+      <c r="B475" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="C475" t="n">
+        <v>42.75</v>
+      </c>
+      <c r="D475" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="E475" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="F475" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="G475" t="n">
+        <v>68.06</v>
+      </c>
+      <c r="H475" t="n">
+        <v>65.28</v>
+      </c>
+      <c r="I475" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="J475" t="n">
+        <v>34.77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-08 (sentiment: 33.88)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J475"/>
+  <dimension ref="A1:J476"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15634,7 +15634,7 @@
         <v>58.5</v>
       </c>
       <c r="E475" t="n">
-        <v>6.78</v>
+        <v>7.06</v>
       </c>
       <c r="F475" t="n">
         <v>4.37</v>
@@ -15646,10 +15646,42 @@
         <v>65.28</v>
       </c>
       <c r="I475" t="n">
-        <v>1.39</v>
+        <v>1.79</v>
       </c>
       <c r="J475" t="n">
-        <v>34.77</v>
+        <v>34.87</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="2" t="n">
+        <v>46273.66666666666</v>
+      </c>
+      <c r="B476" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="C476" t="n">
+        <v>41.65</v>
+      </c>
+      <c r="D476" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="E476" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="F476" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="G476" t="n">
+        <v>63.29</v>
+      </c>
+      <c r="H476" t="n">
+        <v>65.48</v>
+      </c>
+      <c r="I476" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="J476" t="n">
+        <v>33.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-09 (sentiment: 32.69)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J476"/>
+  <dimension ref="A1:J477"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15666,7 +15666,7 @@
         <v>58.5</v>
       </c>
       <c r="E476" t="n">
-        <v>7.12</v>
+        <v>6.97</v>
       </c>
       <c r="F476" t="n">
         <v>4.56</v>
@@ -15678,10 +15678,42 @@
         <v>65.48</v>
       </c>
       <c r="I476" t="n">
-        <v>2.18</v>
+        <v>1.79</v>
       </c>
       <c r="J476" t="n">
-        <v>33.88</v>
+        <v>33.78</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="2" t="n">
+        <v>46274.66666666666</v>
+      </c>
+      <c r="B477" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="C477" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="D477" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="E477" t="n">
+        <v>7.41</v>
+      </c>
+      <c r="F477" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="G477" t="n">
+        <v>57.74</v>
+      </c>
+      <c r="H477" t="n">
+        <v>65.28</v>
+      </c>
+      <c r="I477" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="J477" t="n">
+        <v>32.69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-10 (sentiment: 32.89)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J477"/>
+  <dimension ref="A1:J478"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15698,7 +15698,7 @@
         <v>58.5</v>
       </c>
       <c r="E477" t="n">
-        <v>7.41</v>
+        <v>6.72</v>
       </c>
       <c r="F477" t="n">
         <v>4.76</v>
@@ -15710,10 +15710,42 @@
         <v>65.28</v>
       </c>
       <c r="I477" t="n">
-        <v>2.98</v>
+        <v>0.99</v>
       </c>
       <c r="J477" t="n">
-        <v>32.69</v>
+        <v>32.19</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="2" t="n">
+        <v>46275.66666666666</v>
+      </c>
+      <c r="B478" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="C478" t="n">
+        <v>40.73</v>
+      </c>
+      <c r="D478" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="E478" t="n">
+        <v>7.59</v>
+      </c>
+      <c r="F478" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="G478" t="n">
+        <v>58.13</v>
+      </c>
+      <c r="H478" t="n">
+        <v>65.08</v>
+      </c>
+      <c r="I478" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="J478" t="n">
+        <v>32.89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-11 (sentiment: 32.19)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J478"/>
+  <dimension ref="A1:J479"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15730,7 +15730,7 @@
         <v>58.5</v>
       </c>
       <c r="E478" t="n">
-        <v>7.59</v>
+        <v>6.67</v>
       </c>
       <c r="F478" t="n">
         <v>4.96</v>
@@ -15742,10 +15742,42 @@
         <v>65.08</v>
       </c>
       <c r="I478" t="n">
-        <v>3.37</v>
+        <v>0.99</v>
       </c>
       <c r="J478" t="n">
-        <v>32.89</v>
+        <v>32.29</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="2" t="n">
+        <v>46276.66666666666</v>
+      </c>
+      <c r="B479" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="C479" t="n">
+        <v>40.81</v>
+      </c>
+      <c r="D479" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="E479" t="n">
+        <v>5.58</v>
+      </c>
+      <c r="F479" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="G479" t="n">
+        <v>58.53</v>
+      </c>
+      <c r="H479" t="n">
+        <v>64.88</v>
+      </c>
+      <c r="I479" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J479" t="n">
+        <v>32.19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>